<commit_message>
IFC without dynamic header mapping
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\AmazonDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A18E332-F9B4-4AF3-8571-46772129706E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{284E7E9F-42CB-4294-831D-C92ED0B0DF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -562,6 +562,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -571,9 +574,6 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -961,11 +961,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
       <c r="D1" s="26" t="s">
         <v>53</v>
       </c>
@@ -997,11 +997,11 @@
       <c r="AD1" s="2"/>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="27" t="s">
         <v>49</v>
       </c>
@@ -1037,11 +1037,11 @@
       <c r="AD2" s="2"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
       <c r="D3" s="12" t="s">
         <v>36</v>
       </c>
@@ -1109,42 +1109,42 @@
       <c r="AD4" s="2"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
       <c r="F5" s="37"/>
-      <c r="G5" s="47" t="s">
+      <c r="G5" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="47"/>
-      <c r="I5" s="47"/>
-      <c r="J5" s="47"/>
-      <c r="K5" s="47"/>
-      <c r="L5" s="45" t="s">
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="48"/>
+      <c r="L5" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="45"/>
-      <c r="R5" s="45"/>
-      <c r="S5" s="45"/>
-      <c r="T5" s="45"/>
-      <c r="U5" s="45"/>
-      <c r="V5" s="45"/>
-      <c r="W5" s="45"/>
-      <c r="X5" s="45"/>
-      <c r="Y5" s="45"/>
-      <c r="Z5" s="45"/>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="45"/>
-      <c r="AD5" s="45"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="46"/>
+      <c r="Q5" s="46"/>
+      <c r="R5" s="46"/>
+      <c r="S5" s="46"/>
+      <c r="T5" s="46"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="46"/>
+      <c r="X5" s="46"/>
+      <c r="Y5" s="46"/>
+      <c r="Z5" s="46"/>
+      <c r="AA5" s="46"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="46"/>
+      <c r="AD5" s="46"/>
     </row>
     <row r="6" spans="1:31" s="5" customFormat="1" ht="120.75" x14ac:dyDescent="0.2">
       <c r="A6" s="28" t="s">
@@ -1256,7 +1256,7 @@
         <v>57</v>
       </c>
       <c r="G7" s="43"/>
-      <c r="H7" s="48" t="s">
+      <c r="H7" s="45" t="s">
         <v>60</v>
       </c>
       <c r="I7" s="43"/>

</xml_diff>